<commit_message>
document species interactions conseuences for generation loop
</commit_message>
<xml_diff>
--- a/doc/Manual/Batchmode/InteractionFile.xlsx
+++ b/doc/Manual/Batchmode/InteractionFile.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\theo\github\RangeShifter_batch\doc\Manual\Batchmode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\theop\github\rs_batch_dev\doc\Manual\Batchmode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B60AEA92-F58D-4C95-BE01-D766A85E3926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F782D2CA-9F52-4FB9-8746-DAC5138003FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="2" r:id="rId1"/>
@@ -191,10 +191,10 @@
     <t>one float for each element of ProcessRight</t>
   </si>
   <si>
-    <t xml:space="preserve">One line of input per unique combination of SpeciesLeft, StageLeft, SpeciesRight, StageRight and processes; </t>
-  </si>
-  <si>
     <t>although the reciprocal  interaction (switching left and right) can be specified on a separate line, e.g. to create a two-way directed interaction</t>
+  </si>
+  <si>
+    <t>One line of input per unique combination of SpeciesLeft, StageLeft, SpeciesRight and StageRight;</t>
   </si>
 </sst>
 </file>
@@ -406,8 +406,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Gut" xfId="1" builtinId="26"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -710,25 +710,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.26953125" customWidth="1"/>
-    <col min="2" max="2" width="67.26953125" customWidth="1"/>
-    <col min="3" max="3" width="52.453125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" customWidth="1"/>
+    <col min="2" max="2" width="67.28515625" customWidth="1"/>
+    <col min="3" max="3" width="52.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
@@ -739,7 +739,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
         <v>0</v>
       </c>
@@ -750,7 +750,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
         <v>7</v>
       </c>
@@ -761,7 +761,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
         <v>8</v>
       </c>
@@ -772,7 +772,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>9</v>
       </c>
@@ -783,7 +783,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
         <v>10</v>
       </c>
@@ -794,7 +794,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
         <v>24</v>
       </c>
@@ -805,7 +805,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
         <v>25</v>
       </c>
@@ -816,7 +816,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>11</v>
       </c>
@@ -827,7 +827,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>26</v>
       </c>
@@ -838,7 +838,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>27</v>
       </c>
@@ -849,7 +849,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>28</v>
       </c>
@@ -860,7 +860,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>12</v>
       </c>
@@ -871,7 +871,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>22</v>
       </c>
@@ -882,7 +882,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>13</v>
       </c>
@@ -893,7 +893,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>14</v>
       </c>
@@ -904,7 +904,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
         <v>15</v>
       </c>
@@ -915,7 +915,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
         <v>16</v>
       </c>
@@ -926,7 +926,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
         <v>17</v>
       </c>
@@ -937,7 +937,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>18</v>
       </c>
@@ -948,7 +948,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>19</v>
       </c>
@@ -959,7 +959,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
         <v>20</v>
       </c>
@@ -970,7 +970,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
         <v>21</v>
       </c>
@@ -981,73 +981,73 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C29"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C30"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C31"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C32"/>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33"/>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34"/>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35"/>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C36"/>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37"/>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C38"/>
     </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C39"/>
     </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C40"/>
     </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C41"/>
     </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C42"/>
     </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C43"/>
     </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C44"/>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C45"/>
     </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C46"/>
     </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C47"/>
     </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C48"/>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C49"/>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C50"/>
     </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C51"/>
     </row>
   </sheetData>
@@ -1058,18 +1058,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:V2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="15.81640625" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>

</xml_diff>